<commit_message>
Semana 7: nota de alerta de agotados con la API de Claude
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Inventario" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -427,6 +427,16 @@
           <t>Cantidad</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Precio Un</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Precio Total</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -437,6 +447,12 @@
       <c r="B2" t="n">
         <v>50</v>
       </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>153946.95275</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -447,6 +463,12 @@
       <c r="B3" t="n">
         <v>30</v>
       </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>184736.3433</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -457,6 +479,12 @@
       <c r="B4" t="n">
         <v>0</v>
       </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -466,6 +494,24 @@
       </c>
       <c r="B5" t="n">
         <v>15</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="n">
+        <v>184736.3433</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="n">
+        <v>523419.63935</v>
       </c>
     </row>
   </sheetData>

</xml_diff>